<commit_message>
PEM Capex + LCO Heat
PEM Capex in Datenbanken angepasst, wo das noch nicht der Fall war
LCO Heat in Methane_DAC_Brownfield_Höchst angepasst
Ansonsten Modelldurchläufe
</commit_message>
<xml_diff>
--- a/FischerTropsch_Paper_Michi/FischerTropsch_Naphta_Greenfield_Höchst_MH/Datenbank.xlsx
+++ b/FischerTropsch_Paper_Michi/FischerTropsch_Naphta_Greenfield_Höchst_MH/Datenbank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hem38994\Documents\GitHub\FENES_P2X\FischerTropsch_Paper_Michi\FischerTropsch_Naphta_Greenfield_Höchst_MH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{999458B7-4FA1-4A27-8031-AFFED1CABB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53115BB9-AD9B-465F-933C-9818D2D45B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-4455" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
@@ -1730,6 +1730,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1739,13 +1742,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1754,17 +1754,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1778,8 +1769,17 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2359,7 +2359,7 @@
         <v>26</v>
       </c>
       <c r="E4" s="20">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="F4" t="s">
         <v>83</v>
@@ -3578,10 +3578,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="88" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="90" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="26" t="s">
@@ -3596,7 +3596,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="88"/>
+      <c r="A3" s="89"/>
       <c r="B3" s="85"/>
       <c r="C3" s="13" t="s">
         <v>107</v>
@@ -3610,7 +3610,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="88"/>
+      <c r="A4" s="89"/>
       <c r="B4" s="85"/>
       <c r="C4" s="13" t="s">
         <v>84</v>
@@ -3624,7 +3624,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="88"/>
+      <c r="A5" s="89"/>
       <c r="B5" s="85"/>
       <c r="C5" s="13" t="s">
         <v>138</v>
@@ -3638,7 +3638,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="88"/>
+      <c r="A6" s="89"/>
       <c r="B6" s="85"/>
       <c r="C6" s="13" t="s">
         <v>141</v>
@@ -3652,7 +3652,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="88"/>
+      <c r="A7" s="89"/>
       <c r="B7" s="85"/>
       <c r="C7" s="13" t="s">
         <v>155</v>
@@ -3666,7 +3666,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="88"/>
+      <c r="A8" s="89"/>
       <c r="B8" s="85"/>
       <c r="C8" s="13" t="s">
         <v>196</v>
@@ -3680,7 +3680,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="88"/>
+      <c r="A9" s="89"/>
       <c r="B9" s="85"/>
       <c r="C9" s="13" t="s">
         <v>167</v>
@@ -3694,7 +3694,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="88"/>
+      <c r="A10" s="89"/>
       <c r="B10" s="85"/>
       <c r="C10" s="13" t="s">
         <v>188</v>
@@ -3708,13 +3708,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="88"/>
+      <c r="A11" s="89"/>
       <c r="B11" s="85"/>
       <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="88"/>
-      <c r="B12" s="90" t="s">
+      <c r="A12" s="89"/>
+      <c r="B12" s="100" t="s">
         <v>364</v>
       </c>
       <c r="C12" s="35" t="s">
@@ -3729,7 +3729,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="88"/>
+      <c r="A13" s="89"/>
       <c r="B13" s="91"/>
       <c r="C13" s="13" t="s">
         <v>363</v>
@@ -3743,7 +3743,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="88"/>
+      <c r="A14" s="89"/>
       <c r="B14" s="91"/>
       <c r="C14" s="13" t="s">
         <v>380</v>
@@ -3757,7 +3757,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="88"/>
+      <c r="A15" s="89"/>
       <c r="B15" s="91"/>
       <c r="C15" s="13" t="s">
         <v>139</v>
@@ -3771,7 +3771,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="88"/>
+      <c r="A16" s="89"/>
       <c r="B16" s="91"/>
       <c r="C16" s="13" t="s">
         <v>238</v>
@@ -3785,7 +3785,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="88"/>
+      <c r="A17" s="89"/>
       <c r="B17" s="91"/>
       <c r="C17" s="13" t="s">
         <v>84</v>
@@ -3799,7 +3799,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="88"/>
+      <c r="A18" s="89"/>
       <c r="B18" s="91"/>
       <c r="C18" s="13" t="s">
         <v>141</v>
@@ -3813,7 +3813,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="88"/>
+      <c r="A19" s="89"/>
       <c r="B19" s="91"/>
       <c r="C19" s="13" t="s">
         <v>155</v>
@@ -3827,7 +3827,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="88"/>
+      <c r="A20" s="89"/>
       <c r="B20" s="91"/>
       <c r="C20" s="13" t="s">
         <v>196</v>
@@ -3841,7 +3841,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="88"/>
+      <c r="A21" s="89"/>
       <c r="B21" s="91"/>
       <c r="C21" s="13" t="s">
         <v>167</v>
@@ -3855,7 +3855,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="88"/>
+      <c r="A22" s="89"/>
       <c r="B22" s="91"/>
       <c r="C22" s="13" t="s">
         <v>188</v>
@@ -3869,15 +3869,15 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="88"/>
-      <c r="B23" s="92"/>
+      <c r="A23" s="89"/>
+      <c r="B23" s="101"/>
       <c r="C23" s="36"/>
       <c r="D23" s="36"/>
       <c r="E23" s="37"/>
       <c r="F23" s="36"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="88"/>
+      <c r="A24" s="89"/>
       <c r="B24" s="84" t="s">
         <v>262</v>
       </c>
@@ -3893,7 +3893,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="88"/>
+      <c r="A25" s="89"/>
       <c r="B25" s="85"/>
       <c r="C25" s="13" t="s">
         <v>107</v>
@@ -3907,7 +3907,7 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="88"/>
+      <c r="A26" s="89"/>
       <c r="B26" s="85"/>
       <c r="C26" s="13" t="s">
         <v>84</v>
@@ -3921,7 +3921,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="88"/>
+      <c r="A27" s="89"/>
       <c r="B27" s="85"/>
       <c r="C27" s="13" t="s">
         <v>283</v>
@@ -3935,7 +3935,7 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="88"/>
+      <c r="A28" s="89"/>
       <c r="B28" s="85"/>
       <c r="C28" s="13" t="s">
         <v>141</v>
@@ -3949,7 +3949,7 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="88"/>
+      <c r="A29" s="89"/>
       <c r="B29" s="85"/>
       <c r="C29" s="13" t="s">
         <v>155</v>
@@ -3963,7 +3963,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="88"/>
+      <c r="A30" s="89"/>
       <c r="B30" s="85"/>
       <c r="C30" s="13" t="s">
         <v>196</v>
@@ -3977,7 +3977,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="88"/>
+      <c r="A31" s="89"/>
       <c r="B31" s="85"/>
       <c r="C31" s="13" t="s">
         <v>167</v>
@@ -3991,7 +3991,7 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="88"/>
+      <c r="A32" s="89"/>
       <c r="B32" s="85"/>
       <c r="C32" s="13" t="s">
         <v>188</v>
@@ -4005,7 +4005,7 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="88"/>
+      <c r="A33" s="89"/>
       <c r="B33" s="86"/>
       <c r="C33" s="36"/>
       <c r="D33" s="36"/>
@@ -4013,7 +4013,7 @@
       <c r="F33" s="36"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="88"/>
+      <c r="A34" s="89"/>
       <c r="B34" s="83" t="s">
         <v>229</v>
       </c>
@@ -4029,7 +4029,7 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="88"/>
+      <c r="A35" s="89"/>
       <c r="B35" s="83"/>
       <c r="C35" s="13" t="s">
         <v>107</v>
@@ -4043,7 +4043,7 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="88"/>
+      <c r="A36" s="89"/>
       <c r="B36" s="83"/>
       <c r="C36" s="13" t="s">
         <v>84</v>
@@ -4057,7 +4057,7 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="88"/>
+      <c r="A37" s="89"/>
       <c r="B37" s="83"/>
       <c r="C37" s="13" t="s">
         <v>270</v>
@@ -4071,7 +4071,7 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="88"/>
+      <c r="A38" s="89"/>
       <c r="B38" s="83"/>
       <c r="C38" s="13" t="s">
         <v>248</v>
@@ -4085,7 +4085,7 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="88"/>
+      <c r="A39" s="89"/>
       <c r="B39" s="83"/>
       <c r="C39" s="13" t="s">
         <v>141</v>
@@ -4099,7 +4099,7 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="88"/>
+      <c r="A40" s="89"/>
       <c r="B40" s="83"/>
       <c r="C40" s="13" t="s">
         <v>155</v>
@@ -4113,7 +4113,7 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="88"/>
+      <c r="A41" s="89"/>
       <c r="B41" s="83"/>
       <c r="C41" s="13" t="s">
         <v>196</v>
@@ -4127,7 +4127,7 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="88"/>
+      <c r="A42" s="89"/>
       <c r="B42" s="83"/>
       <c r="C42" s="13" t="s">
         <v>167</v>
@@ -4141,7 +4141,7 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="88"/>
+      <c r="A43" s="89"/>
       <c r="B43" s="83"/>
       <c r="C43" s="13" t="s">
         <v>188</v>
@@ -4155,15 +4155,15 @@
       </c>
     </row>
     <row r="44" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="88"/>
+      <c r="A44" s="89"/>
       <c r="B44" s="83"/>
       <c r="E44" s="33"/>
     </row>
     <row r="45" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="87" t="s">
+      <c r="A45" s="88" t="s">
         <v>71</v>
       </c>
-      <c r="B45" s="96" t="s">
+      <c r="B45" s="103" t="s">
         <v>3</v>
       </c>
       <c r="C45" s="26" t="s">
@@ -4178,7 +4178,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="88"/>
+      <c r="A46" s="89"/>
       <c r="B46" s="83"/>
       <c r="C46" s="13" t="s">
         <v>111</v>
@@ -4192,7 +4192,7 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="88"/>
+      <c r="A47" s="89"/>
       <c r="B47" s="83"/>
       <c r="C47" s="13" t="s">
         <v>135</v>
@@ -4206,7 +4206,7 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="88"/>
+      <c r="A48" s="89"/>
       <c r="B48" s="83"/>
       <c r="C48" s="13" t="s">
         <v>136</v>
@@ -4220,7 +4220,7 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="88"/>
+      <c r="A49" s="89"/>
       <c r="B49" s="83"/>
       <c r="C49" s="13" t="s">
         <v>141</v>
@@ -4234,7 +4234,7 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="88"/>
+      <c r="A50" s="89"/>
       <c r="B50" s="83"/>
       <c r="C50" s="13" t="s">
         <v>155</v>
@@ -4248,7 +4248,7 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="88"/>
+      <c r="A51" s="89"/>
       <c r="B51" s="83"/>
       <c r="C51" s="13" t="s">
         <v>196</v>
@@ -4262,7 +4262,7 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="88"/>
+      <c r="A52" s="89"/>
       <c r="B52" s="83"/>
       <c r="C52" s="13" t="s">
         <v>167</v>
@@ -4276,7 +4276,7 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="88"/>
+      <c r="A53" s="89"/>
       <c r="B53" s="83"/>
       <c r="C53" s="13" t="s">
         <v>188</v>
@@ -4290,15 +4290,15 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="88"/>
-      <c r="B54" s="97"/>
+      <c r="A54" s="89"/>
+      <c r="B54" s="95"/>
       <c r="C54" s="36"/>
       <c r="D54" s="36"/>
       <c r="E54" s="37"/>
       <c r="F54" s="36"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="88"/>
+      <c r="A55" s="89"/>
       <c r="B55" s="83" t="s">
         <v>305</v>
       </c>
@@ -4314,7 +4314,7 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="88"/>
+      <c r="A56" s="89"/>
       <c r="B56" s="83"/>
       <c r="C56" s="13" t="s">
         <v>111</v>
@@ -4328,7 +4328,7 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="88"/>
+      <c r="A57" s="89"/>
       <c r="B57" s="83"/>
       <c r="C57" s="13" t="s">
         <v>135</v>
@@ -4342,7 +4342,7 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="88"/>
+      <c r="A58" s="89"/>
       <c r="B58" s="83"/>
       <c r="C58" s="13" t="s">
         <v>136</v>
@@ -4356,7 +4356,7 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="88"/>
+      <c r="A59" s="89"/>
       <c r="B59" s="83"/>
       <c r="C59" s="13" t="s">
         <v>141</v>
@@ -4370,7 +4370,7 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="88"/>
+      <c r="A60" s="89"/>
       <c r="B60" s="83"/>
       <c r="C60" s="13" t="s">
         <v>155</v>
@@ -4384,7 +4384,7 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="88"/>
+      <c r="A61" s="89"/>
       <c r="B61" s="83"/>
       <c r="C61" s="13" t="s">
         <v>196</v>
@@ -4398,7 +4398,7 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="88"/>
+      <c r="A62" s="89"/>
       <c r="B62" s="83"/>
       <c r="C62" s="13" t="s">
         <v>167</v>
@@ -4412,7 +4412,7 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="88"/>
+      <c r="A63" s="89"/>
       <c r="B63" s="83"/>
       <c r="C63" s="13" t="s">
         <v>188</v>
@@ -4426,12 +4426,12 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="88"/>
-      <c r="B64" s="97"/>
+      <c r="A64" s="89"/>
+      <c r="B64" s="95"/>
       <c r="E64" s="33"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="88"/>
+      <c r="A65" s="89"/>
       <c r="B65" s="94" t="s">
         <v>6</v>
       </c>
@@ -4447,7 +4447,7 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="88"/>
+      <c r="A66" s="89"/>
       <c r="B66" s="83"/>
       <c r="C66" s="13" t="s">
         <v>113</v>
@@ -4461,7 +4461,7 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="88"/>
+      <c r="A67" s="89"/>
       <c r="B67" s="85"/>
       <c r="C67" s="13" t="s">
         <v>111</v>
@@ -4475,7 +4475,7 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="88"/>
+      <c r="A68" s="89"/>
       <c r="B68" s="85"/>
       <c r="C68" s="13" t="s">
         <v>107</v>
@@ -4489,7 +4489,7 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="88"/>
+      <c r="A69" s="89"/>
       <c r="B69" s="85"/>
       <c r="C69" s="13" t="s">
         <v>126</v>
@@ -4503,7 +4503,7 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="88"/>
+      <c r="A70" s="89"/>
       <c r="B70" s="85"/>
       <c r="C70" s="13" t="s">
         <v>127</v>
@@ -4517,7 +4517,7 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="88"/>
+      <c r="A71" s="89"/>
       <c r="B71" s="85"/>
       <c r="C71" s="13" t="s">
         <v>141</v>
@@ -4531,7 +4531,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="88"/>
+      <c r="A72" s="89"/>
       <c r="B72" s="85"/>
       <c r="C72" s="13" t="s">
         <v>155</v>
@@ -4545,7 +4545,7 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="88"/>
+      <c r="A73" s="89"/>
       <c r="B73" s="85"/>
       <c r="C73" s="13" t="s">
         <v>196</v>
@@ -4559,7 +4559,7 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="88"/>
+      <c r="A74" s="89"/>
       <c r="B74" s="85"/>
       <c r="C74" s="13" t="s">
         <v>167</v>
@@ -4573,7 +4573,7 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="88"/>
+      <c r="A75" s="89"/>
       <c r="B75" s="85"/>
       <c r="C75" s="13" t="s">
         <v>188</v>
@@ -4588,17 +4588,17 @@
     </row>
     <row r="76" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="93"/>
-      <c r="B76" s="95"/>
+      <c r="B76" s="102"/>
       <c r="C76" s="40"/>
       <c r="D76" s="40"/>
       <c r="E76" s="41"/>
       <c r="F76" s="40"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="87" t="s">
+      <c r="A77" s="88" t="s">
         <v>72</v>
       </c>
-      <c r="B77" s="89" t="s">
+      <c r="B77" s="90" t="s">
         <v>73</v>
       </c>
       <c r="C77" s="26" t="s">
@@ -4613,7 +4613,7 @@
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="88"/>
+      <c r="A78" s="89"/>
       <c r="B78" s="85"/>
       <c r="C78" s="13" t="s">
         <v>153</v>
@@ -4627,12 +4627,12 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="88"/>
+      <c r="A79" s="89"/>
       <c r="B79" s="86"/>
       <c r="E79" s="31"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="88"/>
+      <c r="A80" s="89"/>
       <c r="B80" s="94" t="s">
         <v>4</v>
       </c>
@@ -4648,7 +4648,7 @@
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="88"/>
+      <c r="A81" s="89"/>
       <c r="B81" s="83"/>
       <c r="C81" s="13" t="s">
         <v>107</v>
@@ -4662,7 +4662,7 @@
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="88"/>
+      <c r="A82" s="89"/>
       <c r="B82" s="83"/>
       <c r="C82" s="13" t="s">
         <v>122</v>
@@ -4676,7 +4676,7 @@
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="88"/>
+      <c r="A83" s="89"/>
       <c r="B83" s="83"/>
       <c r="C83" s="13" t="s">
         <v>141</v>
@@ -4690,7 +4690,7 @@
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="88"/>
+      <c r="A84" s="89"/>
       <c r="B84" s="83"/>
       <c r="C84" s="13" t="s">
         <v>155</v>
@@ -4704,7 +4704,7 @@
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="88"/>
+      <c r="A85" s="89"/>
       <c r="B85" s="83"/>
       <c r="C85" s="13" t="s">
         <v>161</v>
@@ -4718,7 +4718,7 @@
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="88"/>
+      <c r="A86" s="89"/>
       <c r="B86" s="83"/>
       <c r="C86" s="13" t="s">
         <v>196</v>
@@ -4732,7 +4732,7 @@
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="88"/>
+      <c r="A87" s="89"/>
       <c r="B87" s="83"/>
       <c r="C87" s="13" t="s">
         <v>167</v>
@@ -4746,7 +4746,7 @@
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="88"/>
+      <c r="A88" s="89"/>
       <c r="B88" s="83"/>
       <c r="C88" s="13" t="s">
         <v>188</v>
@@ -4760,11 +4760,11 @@
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="88"/>
-      <c r="B89" s="97"/>
+      <c r="A89" s="89"/>
+      <c r="B89" s="95"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="88"/>
+      <c r="A90" s="89"/>
       <c r="B90" s="94" t="s">
         <v>5</v>
       </c>
@@ -4780,7 +4780,7 @@
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="88"/>
+      <c r="A91" s="89"/>
       <c r="B91" s="83"/>
       <c r="C91" s="13" t="s">
         <v>108</v>
@@ -4794,7 +4794,7 @@
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="88"/>
+      <c r="A92" s="89"/>
       <c r="B92" s="83"/>
       <c r="C92" s="13" t="s">
         <v>120</v>
@@ -4808,7 +4808,7 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="88"/>
+      <c r="A93" s="89"/>
       <c r="B93" s="83"/>
       <c r="C93" s="13" t="s">
         <v>141</v>
@@ -4822,7 +4822,7 @@
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="88"/>
+      <c r="A94" s="89"/>
       <c r="B94" s="83"/>
       <c r="C94" s="13" t="s">
         <v>155</v>
@@ -4836,7 +4836,7 @@
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="88"/>
+      <c r="A95" s="89"/>
       <c r="B95" s="83"/>
       <c r="C95" s="13" t="s">
         <v>161</v>
@@ -4850,7 +4850,7 @@
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="88"/>
+      <c r="A96" s="89"/>
       <c r="B96" s="83"/>
       <c r="C96" s="13" t="s">
         <v>196</v>
@@ -4864,7 +4864,7 @@
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="88"/>
+      <c r="A97" s="89"/>
       <c r="B97" s="83"/>
       <c r="C97" s="13" t="s">
         <v>167</v>
@@ -4878,7 +4878,7 @@
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="88"/>
+      <c r="A98" s="89"/>
       <c r="B98" s="83"/>
       <c r="C98" s="13" t="s">
         <v>188</v>
@@ -4893,13 +4893,13 @@
     </row>
     <row r="99" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A99" s="93"/>
-      <c r="B99" s="99"/>
+      <c r="B99" s="96"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="87" t="s">
+      <c r="A100" s="88" t="s">
         <v>76</v>
       </c>
-      <c r="B100" s="89" t="s">
+      <c r="B100" s="90" t="s">
         <v>73</v>
       </c>
       <c r="C100" s="26" t="s">
@@ -4914,7 +4914,7 @@
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="88"/>
+      <c r="A101" s="89"/>
       <c r="B101" s="85"/>
       <c r="C101" s="13" t="s">
         <v>228</v>
@@ -4928,7 +4928,7 @@
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="88"/>
+      <c r="A102" s="89"/>
       <c r="B102" s="85"/>
       <c r="C102" s="13" t="s">
         <v>150</v>
@@ -4942,7 +4942,7 @@
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="88"/>
+      <c r="A103" s="89"/>
       <c r="B103" s="86"/>
       <c r="C103" s="36"/>
       <c r="D103" s="36"/>
@@ -4950,7 +4950,7 @@
       <c r="F103" s="36"/>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="88"/>
+      <c r="A104" s="89"/>
       <c r="B104" s="84" t="s">
         <v>292</v>
       </c>
@@ -4966,7 +4966,7 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="88"/>
+      <c r="A105" s="89"/>
       <c r="B105" s="85"/>
       <c r="C105" s="13" t="s">
         <v>297</v>
@@ -4980,7 +4980,7 @@
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="88"/>
+      <c r="A106" s="89"/>
       <c r="B106" s="85"/>
       <c r="C106" s="13" t="s">
         <v>298</v>
@@ -4994,12 +4994,12 @@
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="88"/>
+      <c r="A107" s="89"/>
       <c r="B107" s="86"/>
       <c r="E107" s="33"/>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="88"/>
+      <c r="A108" s="89"/>
       <c r="B108" s="84" t="s">
         <v>79</v>
       </c>
@@ -5015,7 +5015,7 @@
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="88"/>
+      <c r="A109" s="89"/>
       <c r="B109" s="85"/>
       <c r="C109" s="13" t="s">
         <v>151</v>
@@ -5029,7 +5029,7 @@
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="88"/>
+      <c r="A110" s="89"/>
       <c r="B110" s="86"/>
       <c r="C110" s="36"/>
       <c r="D110" s="36"/>
@@ -5037,8 +5037,8 @@
       <c r="F110" s="36"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="88"/>
-      <c r="B111" s="100" t="s">
+      <c r="A111" s="89"/>
+      <c r="B111" s="97" t="s">
         <v>371</v>
       </c>
       <c r="C111" s="35" t="s">
@@ -5053,8 +5053,8 @@
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" s="88"/>
-      <c r="B112" s="101"/>
+      <c r="A112" s="89"/>
+      <c r="B112" s="98"/>
       <c r="C112" s="13" t="s">
         <v>376</v>
       </c>
@@ -5067,15 +5067,15 @@
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="88"/>
-      <c r="B113" s="102"/>
+      <c r="A113" s="89"/>
+      <c r="B113" s="99"/>
       <c r="C113" s="36"/>
       <c r="D113" s="36"/>
       <c r="E113" s="37"/>
       <c r="F113" s="36"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A114" s="88"/>
+      <c r="A114" s="89"/>
       <c r="B114" s="91" t="s">
         <v>331</v>
       </c>
@@ -5091,7 +5091,7 @@
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A115" s="88"/>
+      <c r="A115" s="89"/>
       <c r="B115" s="91"/>
       <c r="C115" s="13" t="s">
         <v>362</v>
@@ -5106,17 +5106,17 @@
     </row>
     <row r="116" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A116" s="93"/>
-      <c r="B116" s="98"/>
+      <c r="B116" s="92"/>
       <c r="C116" s="40"/>
       <c r="D116" s="40"/>
       <c r="E116" s="41"/>
       <c r="F116" s="40"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" s="87" t="s">
+      <c r="A117" s="88" t="s">
         <v>163</v>
       </c>
-      <c r="B117" s="89" t="s">
+      <c r="B117" s="90" t="s">
         <v>13</v>
       </c>
       <c r="C117" s="26" t="s">
@@ -5131,7 +5131,7 @@
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" s="88"/>
+      <c r="A118" s="89"/>
       <c r="B118" s="85"/>
       <c r="C118" s="13" t="s">
         <v>174</v>
@@ -5144,7 +5144,7 @@
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="88"/>
+      <c r="A119" s="89"/>
       <c r="B119" s="86"/>
       <c r="C119" s="36"/>
       <c r="D119" s="36"/>
@@ -5152,7 +5152,7 @@
       <c r="F119" s="36"/>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" s="88"/>
+      <c r="A120" s="89"/>
       <c r="B120" s="84" t="s">
         <v>183</v>
       </c>
@@ -5167,7 +5167,7 @@
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121" s="88"/>
+      <c r="A121" s="89"/>
       <c r="B121" s="85"/>
       <c r="C121" s="13" t="s">
         <v>181</v>
@@ -5180,7 +5180,7 @@
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" s="88"/>
+      <c r="A122" s="89"/>
       <c r="B122" s="85"/>
       <c r="C122" s="13" t="s">
         <v>177</v>
@@ -5193,7 +5193,7 @@
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A123" s="88"/>
+      <c r="A123" s="89"/>
       <c r="B123" s="85"/>
       <c r="C123" s="13" t="s">
         <v>179</v>
@@ -5206,7 +5206,7 @@
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A124" s="88"/>
+      <c r="A124" s="89"/>
       <c r="B124" s="85"/>
       <c r="C124" s="13" t="s">
         <v>182</v>
@@ -5219,7 +5219,7 @@
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A125" s="88"/>
+      <c r="A125" s="89"/>
       <c r="B125" s="85"/>
       <c r="C125" s="13" t="s">
         <v>191</v>
@@ -5232,11 +5232,11 @@
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" s="88"/>
+      <c r="A126" s="89"/>
       <c r="B126" s="86"/>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" s="88"/>
+      <c r="A127" s="89"/>
       <c r="B127" s="84" t="s">
         <v>206</v>
       </c>
@@ -5252,7 +5252,7 @@
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" s="88"/>
+      <c r="A128" s="89"/>
       <c r="B128" s="85"/>
       <c r="C128" s="13" t="s">
         <v>204</v>
@@ -5265,7 +5265,7 @@
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="88"/>
+      <c r="A129" s="89"/>
       <c r="B129" s="85"/>
       <c r="C129" s="13" t="s">
         <v>215</v>
@@ -5278,7 +5278,7 @@
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="88"/>
+      <c r="A130" s="89"/>
       <c r="B130" s="85"/>
       <c r="C130" s="13" t="s">
         <v>205</v>
@@ -5291,7 +5291,7 @@
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="88"/>
+      <c r="A131" s="89"/>
       <c r="B131" s="85"/>
       <c r="C131" s="13" t="s">
         <v>300</v>
@@ -5304,7 +5304,7 @@
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="88"/>
+      <c r="A132" s="89"/>
       <c r="B132" s="85"/>
       <c r="C132" s="44" t="s">
         <v>324</v>
@@ -5318,7 +5318,7 @@
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="88"/>
+      <c r="A133" s="89"/>
       <c r="B133" s="85"/>
       <c r="C133" s="44" t="s">
         <v>326</v>
@@ -5332,7 +5332,7 @@
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="88"/>
+      <c r="A134" s="89"/>
       <c r="B134" s="85"/>
       <c r="C134" s="13" t="s">
         <v>217</v>
@@ -5345,7 +5345,7 @@
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="88"/>
+      <c r="A135" s="89"/>
       <c r="B135" s="85"/>
       <c r="C135" s="13" t="s">
         <v>221</v>
@@ -5358,7 +5358,7 @@
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="88"/>
+      <c r="A136" s="89"/>
       <c r="B136" s="85"/>
       <c r="C136" s="13" t="s">
         <v>202</v>
@@ -5371,7 +5371,7 @@
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137" s="88"/>
+      <c r="A137" s="89"/>
       <c r="B137" s="85"/>
       <c r="C137" s="44" t="s">
         <v>249</v>
@@ -5385,7 +5385,7 @@
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A138" s="88"/>
+      <c r="A138" s="89"/>
       <c r="B138" s="85"/>
       <c r="C138" s="44" t="s">
         <v>383</v>
@@ -5399,7 +5399,7 @@
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A139" s="88"/>
+      <c r="A139" s="89"/>
       <c r="B139" s="85"/>
       <c r="C139" s="44" t="s">
         <v>365</v>
@@ -5413,7 +5413,7 @@
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A140" s="88"/>
+      <c r="A140" s="89"/>
       <c r="B140" s="85"/>
       <c r="C140" s="44" t="s">
         <v>385</v>
@@ -5427,7 +5427,7 @@
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A141" s="88"/>
+      <c r="A141" s="89"/>
       <c r="B141" s="86"/>
       <c r="C141" s="44"/>
       <c r="D141" s="44"/>
@@ -5435,7 +5435,7 @@
       <c r="F141" s="44"/>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142" s="88"/>
+      <c r="A142" s="89"/>
       <c r="B142" s="84" t="s">
         <v>222</v>
       </c>
@@ -5451,7 +5451,7 @@
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143" s="88"/>
+      <c r="A143" s="89"/>
       <c r="B143" s="85"/>
       <c r="C143" s="13" t="s">
         <v>302</v>
@@ -5464,7 +5464,7 @@
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A144" s="88"/>
+      <c r="A144" s="89"/>
       <c r="B144" s="85"/>
       <c r="C144" s="13" t="s">
         <v>225</v>
@@ -5477,7 +5477,7 @@
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A145" s="88"/>
+      <c r="A145" s="89"/>
       <c r="B145" s="85"/>
       <c r="C145" s="44" t="s">
         <v>251</v>
@@ -5491,7 +5491,7 @@
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A146" s="88"/>
+      <c r="A146" s="89"/>
       <c r="B146" s="85"/>
       <c r="C146" s="44" t="s">
         <v>366</v>
@@ -5505,7 +5505,7 @@
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A147" s="88"/>
+      <c r="A147" s="89"/>
       <c r="B147" s="86"/>
       <c r="C147" s="36"/>
       <c r="D147" s="36"/>
@@ -5513,8 +5513,8 @@
       <c r="F147" s="36"/>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A148" s="88"/>
-      <c r="B148" s="103" t="s">
+      <c r="A148" s="89"/>
+      <c r="B148" s="87" t="s">
         <v>386</v>
       </c>
       <c r="C148" s="13" t="s">
@@ -5528,8 +5528,8 @@
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A149" s="88"/>
-      <c r="B149" s="103"/>
+      <c r="A149" s="89"/>
+      <c r="B149" s="87"/>
       <c r="C149" s="13" t="s">
         <v>388</v>
       </c>
@@ -5542,12 +5542,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B142:B147"/>
-    <mergeCell ref="B148:B149"/>
-    <mergeCell ref="A117:A149"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="B127:B141"/>
-    <mergeCell ref="B120:B126"/>
+    <mergeCell ref="A2:A44"/>
+    <mergeCell ref="B2:B11"/>
+    <mergeCell ref="B12:B23"/>
+    <mergeCell ref="B34:B44"/>
+    <mergeCell ref="A45:A76"/>
+    <mergeCell ref="B65:B76"/>
+    <mergeCell ref="B24:B33"/>
+    <mergeCell ref="B45:B54"/>
+    <mergeCell ref="B55:B64"/>
     <mergeCell ref="B114:B116"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="A77:A99"/>
@@ -5558,15 +5561,12 @@
     <mergeCell ref="B104:B107"/>
     <mergeCell ref="B108:B110"/>
     <mergeCell ref="B111:B113"/>
-    <mergeCell ref="A2:A44"/>
-    <mergeCell ref="B2:B11"/>
-    <mergeCell ref="B12:B23"/>
-    <mergeCell ref="B34:B44"/>
-    <mergeCell ref="A45:A76"/>
-    <mergeCell ref="B65:B76"/>
-    <mergeCell ref="B24:B33"/>
-    <mergeCell ref="B45:B54"/>
-    <mergeCell ref="B55:B64"/>
+    <mergeCell ref="B142:B147"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="A117:A149"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="B127:B141"/>
+    <mergeCell ref="B120:B126"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>